<commit_message>
update sample import barang masuk
</commit_message>
<xml_diff>
--- a/assets/sample/test_import_barang_masuk.xlsx
+++ b/assets/sample/test_import_barang_masuk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\keuanganApp\assets\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256C120E-8DB8-4BE5-A0F6-520136074D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A70EBE-37EF-4D79-A86F-B370C19C1656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{59848987-8667-4A33-BB81-346273598465}"/>
   </bookViews>
@@ -34,33 +34,66 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>kode_barang</t>
-  </si>
-  <si>
-    <t>nama_barang</t>
-  </si>
-  <si>
-    <t>jumlah</t>
-  </si>
-  <si>
-    <t>harga_beli</t>
-  </si>
-  <si>
-    <t>tanggal_transaksi</t>
-  </si>
-  <si>
-    <t>WB-803</t>
-  </si>
-  <si>
-    <t>PENGHAPUS PAPAN TULIS</t>
-  </si>
-  <si>
-    <t>CM07</t>
-  </si>
-  <si>
-    <t>Web Cam JQVITEK</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+  <si>
+    <t>MIIND</t>
+  </si>
+  <si>
+    <t>Indomie Goreng</t>
+  </si>
+  <si>
+    <t>Makanan</t>
+  </si>
+  <si>
+    <t>S4G</t>
+  </si>
+  <si>
+    <t>Sosis</t>
+  </si>
+  <si>
+    <t>SWSPRT</t>
+  </si>
+  <si>
+    <t>Sprite 150 ml</t>
+  </si>
+  <si>
+    <t>Minuman</t>
+  </si>
+  <si>
+    <t>Kode Barang</t>
+  </si>
+  <si>
+    <t>Merk</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Isi</t>
+  </si>
+  <si>
+    <t>Jumlah</t>
+  </si>
+  <si>
+    <t>Harga Beli</t>
+  </si>
+  <si>
+    <t>Tanggal Transaksi</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>No Mitra</t>
+  </si>
+  <si>
+    <t>Indofood</t>
+  </si>
+  <si>
+    <t>Pak Suharjo</t>
+  </si>
+  <si>
+    <t>Garuda</t>
   </si>
 </sst>
 </file>
@@ -413,65 +446,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8D1893F-5EA9-4DCE-B18D-DC2A8D071494}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" style="1" customWidth="1"/>
+    <col min="3" max="4" width="22.5546875" customWidth="1"/>
+    <col min="7" max="7" width="21" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2">
+        <v>50</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <v>100000</v>
+      </c>
+      <c r="G2" s="1">
+        <f ca="1">NOW()</f>
+        <v>45647.539496759258</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2">
+        <v>10293091820</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>30000</v>
+      </c>
+      <c r="G3" s="1">
+        <f ca="1">NOW()</f>
+        <v>45647.539496759258</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3">
+        <v>93840291920</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>15</v>
+      </c>
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="D2">
-        <v>7500</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="F4">
+        <v>150000</v>
+      </c>
+      <c r="G4" s="1">
         <f ca="1">NOW()</f>
-        <v>45544.336260648146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>100000</v>
-      </c>
-      <c r="E3" s="1">
-        <f ca="1">NOW()</f>
-        <v>45544.336260648146</v>
+        <v>45647.539496759258</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4">
+        <v>40948092301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>